<commit_message>
Update Sprint 5 backlog
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_5_Backlog.xlsx
+++ b/documentation/scrum/Sprint_5_Backlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imashai\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC70D85-0FDC-4E58-8A36-21F8E392EB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{5CC70D85-0FDC-4E58-8A36-21F8E392EB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A75303A-2E6D-478D-BF65-691F16070FCC}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="124">
   <si>
     <t>CIS4014-N Interactive Visualisation – Group 4 | Sprint 5 – Week 05</t>
   </si>
@@ -388,14 +388,17 @@
     <t>https://github.com/inkymello/group4-interactive-visualisation/tree/main/documentation/meetings</t>
   </si>
   <si>
-    <t>vvv</t>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/meetings/Final_Team_Review.docx</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/documentation/scrum/Final_Scrum_Review.docx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,21 +444,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -478,7 +466,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -499,12 +487,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1166,8 +1148,8 @@
       <c r="H23" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I23" s="11" t="s">
-        <v>122</v>
+      <c r="I23" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.35">
@@ -1369,7 +1351,7 @@
       <c r="H30" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="I30" s="10" t="s">
+      <c r="I30" s="6" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1407,11 +1389,13 @@
   <hyperlinks>
     <hyperlink ref="I26" r:id="rId1" xr:uid="{B386B54F-0DAA-42A4-81EE-9143593C8E1C}"/>
     <hyperlink ref="I27" r:id="rId2" xr:uid="{28156D17-4A5A-4F56-8313-833A7082A7E9}"/>
+    <hyperlink ref="I30" r:id="rId3" xr:uid="{6910F0F7-E6A4-47C6-B4F1-6C567E4EFDAF}"/>
+    <hyperlink ref="I23" r:id="rId4" xr:uid="{B3C38439-4C81-4284-B1AD-D449C8240EE8}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>